<commit_message>
feat: Add document processing test case for document 001598405, including input PDF, generated prompts, and extracted data, with corresponding updates to main, prompts, and pipeline logic.
</commit_message>
<xml_diff>
--- a/data/out/動作確認/1-1_Python版.xlsx
+++ b/data/out/動作確認/1-1_Python版.xlsx
@@ -7,10 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Sheet1'!$A$1:$AG$48</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Sheet'!$A$1:$AG$50</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -42,7 +42,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="20">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -72,6 +72,7 @@
       <right style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border/>
     <border>
       <left style="thin"/>
       <right style="thin"/>
@@ -97,59 +98,11 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right/>
-      <top/>
-      <bottom style="thin"/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin"/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin"/>
-      <top/>
-      <bottom style="thin"/>
-    </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top/>
-      <bottom style="thin"/>
-    </border>
-    <border>
-      <left style="thin"/>
-      <right/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -169,9 +122,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -181,28 +131,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -568,7 +508,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="F1:AG50"/>
+  <dimension ref="F3:AG50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.53" customWidth="1" min="1" max="1"/>
@@ -607,127 +547,200 @@
     <col width="2.53" customWidth="1" min="34" max="34"/>
     <col width="2.53" customWidth="1" min="35" max="35"/>
     <col width="2.53" customWidth="1" min="36" max="36"/>
+    <col width="2.53" customWidth="1" min="37" max="37"/>
+    <col width="2.53" customWidth="1" min="38" max="38"/>
+    <col width="2.53" customWidth="1" min="39" max="39"/>
+    <col width="2.53" customWidth="1" min="40" max="40"/>
+    <col width="2.53" customWidth="1" min="41" max="41"/>
+    <col width="2.53" customWidth="1" min="42" max="42"/>
+    <col width="2.53" customWidth="1" min="43" max="43"/>
+    <col width="2.53" customWidth="1" min="44" max="44"/>
+    <col width="2.53" customWidth="1" min="45" max="45"/>
+    <col width="2.53" customWidth="1" min="46" max="46"/>
+    <col width="2.53" customWidth="1" min="47" max="47"/>
+    <col width="2.53" customWidth="1" min="48" max="48"/>
+    <col width="2.53" customWidth="1" min="49" max="49"/>
+    <col width="2.53" customWidth="1" min="50" max="50"/>
+    <col width="2.53" customWidth="1" min="51" max="51"/>
+    <col width="2.53" customWidth="1" min="52" max="52"/>
+    <col width="2.53" customWidth="1" min="53" max="53"/>
+    <col width="2.53" customWidth="1" min="54" max="54"/>
+    <col width="2.53" customWidth="1" min="55" max="55"/>
+    <col width="2.53" customWidth="1" min="56" max="56"/>
+    <col width="2.53" customWidth="1" min="57" max="57"/>
+    <col width="2.53" customWidth="1" min="58" max="58"/>
+    <col width="2.53" customWidth="1" min="59" max="59"/>
+    <col width="2.53" customWidth="1" min="60" max="60"/>
+    <col width="2.53" customWidth="1" min="61" max="61"/>
+    <col width="2.53" customWidth="1" min="62" max="62"/>
+    <col width="2.53" customWidth="1" min="63" max="63"/>
+    <col width="2.53" customWidth="1" min="64" max="64"/>
+    <col width="2.53" customWidth="1" min="65" max="65"/>
+    <col width="2.53" customWidth="1" min="66" max="66"/>
+    <col width="2.53" customWidth="1" min="67" max="67"/>
+    <col width="2.53" customWidth="1" min="68" max="68"/>
+    <col width="2.53" customWidth="1" min="69" max="69"/>
+    <col width="2.53" customWidth="1" min="70" max="70"/>
+    <col width="2.53" customWidth="1" min="71" max="71"/>
+    <col width="2.53" customWidth="1" min="72" max="72"/>
+    <col width="2.53" customWidth="1" min="73" max="73"/>
+    <col width="2.53" customWidth="1" min="74" max="74"/>
+    <col width="2.53" customWidth="1" min="75" max="75"/>
+    <col width="2.53" customWidth="1" min="76" max="76"/>
+    <col width="2.53" customWidth="1" min="77" max="77"/>
+    <col width="2.53" customWidth="1" min="78" max="78"/>
+    <col width="2.53" customWidth="1" min="79" max="79"/>
+    <col width="2.53" customWidth="1" min="80" max="80"/>
+    <col width="2.53" customWidth="1" min="81" max="81"/>
+    <col width="2.53" customWidth="1" min="82" max="82"/>
+    <col width="2.53" customWidth="1" min="83" max="83"/>
+    <col width="2.53" customWidth="1" min="84" max="84"/>
+    <col width="2.53" customWidth="1" min="85" max="85"/>
+    <col width="2.53" customWidth="1" min="86" max="86"/>
+    <col width="2.53" customWidth="1" min="87" max="87"/>
+    <col width="2.53" customWidth="1" min="88" max="88"/>
+    <col width="2.53" customWidth="1" min="89" max="89"/>
+    <col width="2.53" customWidth="1" min="90" max="90"/>
+    <col width="2.53" customWidth="1" min="91" max="91"/>
+    <col width="2.53" customWidth="1" min="92" max="92"/>
+    <col width="2.53" customWidth="1" min="93" max="93"/>
+    <col width="2.53" customWidth="1" min="94" max="94"/>
+    <col width="2.53" customWidth="1" min="95" max="95"/>
+    <col width="2.53" customWidth="1" min="96" max="96"/>
+    <col width="2.53" customWidth="1" min="97" max="97"/>
+    <col width="2.53" customWidth="1" min="98" max="98"/>
+    <col width="2.53" customWidth="1" min="99" max="99"/>
+    <col width="2.53" customWidth="1" min="100" max="100"/>
+    <col width="2.53" customWidth="1" min="101" max="101"/>
+    <col width="2.53" customWidth="1" min="102" max="102"/>
+    <col width="2.53" customWidth="1" min="103" max="103"/>
+    <col width="2.53" customWidth="1" min="104" max="104"/>
+    <col width="2.53" customWidth="1" min="105" max="105"/>
+    <col width="2.53" customWidth="1" min="106" max="106"/>
+    <col width="2.53" customWidth="1" min="107" max="107"/>
+    <col width="2.53" customWidth="1" min="108" max="108"/>
+    <col width="2.53" customWidth="1" min="109" max="109"/>
+    <col width="2.53" customWidth="1" min="110" max="110"/>
+    <col width="2.53" customWidth="1" min="111" max="111"/>
+    <col width="2.53" customWidth="1" min="112" max="112"/>
+    <col width="2.53" customWidth="1" min="113" max="113"/>
+    <col width="2.53" customWidth="1" min="114" max="114"/>
+    <col width="2.53" customWidth="1" min="115" max="115"/>
+    <col width="2.53" customWidth="1" min="116" max="116"/>
+    <col width="2.53" customWidth="1" min="117" max="117"/>
+    <col width="2.53" customWidth="1" min="118" max="118"/>
+    <col width="2.53" customWidth="1" min="119" max="119"/>
+    <col width="2.53" customWidth="1" min="120" max="120"/>
+    <col width="2.53" customWidth="1" min="121" max="121"/>
+    <col width="2.53" customWidth="1" min="122" max="122"/>
+    <col width="2.53" customWidth="1" min="123" max="123"/>
+    <col width="2.53" customWidth="1" min="124" max="124"/>
+    <col width="2.53" customWidth="1" min="125" max="125"/>
+    <col width="2.53" customWidth="1" min="126" max="126"/>
+    <col width="2.53" customWidth="1" min="127" max="127"/>
+    <col width="2.53" customWidth="1" min="128" max="128"/>
+    <col width="2.53" customWidth="1" min="129" max="129"/>
+    <col width="2.53" customWidth="1" min="130" max="130"/>
+    <col width="2.53" customWidth="1" min="131" max="131"/>
+    <col width="2.53" customWidth="1" min="132" max="132"/>
+    <col width="2.53" customWidth="1" min="133" max="133"/>
+    <col width="2.53" customWidth="1" min="134" max="134"/>
+    <col width="2.53" customWidth="1" min="135" max="135"/>
+    <col width="2.53" customWidth="1" min="136" max="136"/>
+    <col width="2.53" customWidth="1" min="137" max="137"/>
+    <col width="2.53" customWidth="1" min="138" max="138"/>
+    <col width="2.53" customWidth="1" min="139" max="139"/>
+    <col width="2.53" customWidth="1" min="140" max="140"/>
+    <col width="2.53" customWidth="1" min="141" max="141"/>
+    <col width="2.53" customWidth="1" min="142" max="142"/>
+    <col width="2.53" customWidth="1" min="143" max="143"/>
+    <col width="2.53" customWidth="1" min="144" max="144"/>
+    <col width="2.53" customWidth="1" min="145" max="145"/>
+    <col width="2.53" customWidth="1" min="146" max="146"/>
+    <col width="2.53" customWidth="1" min="147" max="147"/>
+    <col width="2.53" customWidth="1" min="148" max="148"/>
+    <col width="2.53" customWidth="1" min="149" max="149"/>
+    <col width="2.53" customWidth="1" min="150" max="150"/>
+    <col width="2.53" customWidth="1" min="151" max="151"/>
+    <col width="2.53" customWidth="1" min="152" max="152"/>
+    <col width="2.53" customWidth="1" min="153" max="153"/>
+    <col width="2.53" customWidth="1" min="154" max="154"/>
+    <col width="2.53" customWidth="1" min="155" max="155"/>
+    <col width="2.53" customWidth="1" min="156" max="156"/>
+    <col width="2.53" customWidth="1" min="157" max="157"/>
+    <col width="2.53" customWidth="1" min="158" max="158"/>
+    <col width="2.53" customWidth="1" min="159" max="159"/>
+    <col width="2.53" customWidth="1" min="160" max="160"/>
+    <col width="2.53" customWidth="1" min="161" max="161"/>
+    <col width="2.53" customWidth="1" min="162" max="162"/>
+    <col width="2.53" customWidth="1" min="163" max="163"/>
+    <col width="2.53" customWidth="1" min="164" max="164"/>
+    <col width="2.53" customWidth="1" min="165" max="165"/>
+    <col width="2.53" customWidth="1" min="166" max="166"/>
+    <col width="2.53" customWidth="1" min="167" max="167"/>
+    <col width="2.53" customWidth="1" min="168" max="168"/>
+    <col width="2.53" customWidth="1" min="169" max="169"/>
+    <col width="2.53" customWidth="1" min="170" max="170"/>
+    <col width="2.53" customWidth="1" min="171" max="171"/>
+    <col width="2.53" customWidth="1" min="172" max="172"/>
+    <col width="2.53" customWidth="1" min="173" max="173"/>
+    <col width="2.53" customWidth="1" min="174" max="174"/>
+    <col width="2.53" customWidth="1" min="175" max="175"/>
+    <col width="2.53" customWidth="1" min="176" max="176"/>
+    <col width="2.53" customWidth="1" min="177" max="177"/>
+    <col width="2.53" customWidth="1" min="178" max="178"/>
+    <col width="2.53" customWidth="1" min="179" max="179"/>
+    <col width="2.53" customWidth="1" min="180" max="180"/>
+    <col width="2.53" customWidth="1" min="181" max="181"/>
+    <col width="2.53" customWidth="1" min="182" max="182"/>
+    <col width="2.53" customWidth="1" min="183" max="183"/>
+    <col width="2.53" customWidth="1" min="184" max="184"/>
+    <col width="2.53" customWidth="1" min="185" max="185"/>
+    <col width="2.53" customWidth="1" min="186" max="186"/>
+    <col width="2.53" customWidth="1" min="187" max="187"/>
+    <col width="2.53" customWidth="1" min="188" max="188"/>
+    <col width="2.53" customWidth="1" min="189" max="189"/>
+    <col width="2.53" customWidth="1" min="190" max="190"/>
+    <col width="2.53" customWidth="1" min="191" max="191"/>
+    <col width="2.53" customWidth="1" min="192" max="192"/>
+    <col width="2.53" customWidth="1" min="193" max="193"/>
+    <col width="2.53" customWidth="1" min="194" max="194"/>
+    <col width="2.53" customWidth="1" min="195" max="195"/>
+    <col width="2.53" customWidth="1" min="196" max="196"/>
+    <col width="2.53" customWidth="1" min="197" max="197"/>
+    <col width="2.53" customWidth="1" min="198" max="198"/>
+    <col width="2.53" customWidth="1" min="199" max="199"/>
   </cols>
   <sheetData>
-    <row r="1" ht="17.01" customHeight="1">
-      <c r="F1" s="1" t="inlineStr">
+    <row r="1" ht="17.01" customHeight="1"/>
+    <row r="2" ht="17.01" customHeight="1"/>
+    <row r="3" ht="17.01" customHeight="1">
+      <c r="F3" s="1" t="inlineStr">
         <is>
           <t>表１－１</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I3" s="1" t="inlineStr">
         <is>
           <t>管理施設数（国土交通省管理分）</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="17.01" customHeight="1">
-      <c r="AA2" s="2" t="inlineStr">
+    <row r="4" ht="17.01" customHeight="1">
+      <c r="AA4" s="2" t="inlineStr">
         <is>
           <t>平成30年3月31日時点</t>
         </is>
       </c>
-    </row>
-    <row r="3" ht="17.01" customHeight="1">
-      <c r="F3" s="3" t="n"/>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>所在する都道府県</t>
-        </is>
-      </c>
-      <c r="H3" s="5" t="n"/>
-      <c r="I3" s="5" t="n"/>
-      <c r="J3" s="5" t="n"/>
-      <c r="K3" s="5" t="n"/>
-      <c r="L3" s="5" t="n"/>
-      <c r="M3" s="3" t="n"/>
-      <c r="N3" s="5" t="n"/>
-      <c r="O3" s="4" t="inlineStr">
-        <is>
-          <t>橋梁</t>
-        </is>
-      </c>
-      <c r="P3" s="5" t="n"/>
-      <c r="Q3" s="5" t="n"/>
-      <c r="R3" s="5" t="n"/>
-      <c r="S3" s="3" t="n"/>
-      <c r="T3" s="5" t="n"/>
-      <c r="U3" s="5" t="n"/>
-      <c r="V3" s="4" t="inlineStr">
-        <is>
-          <t>トンネル</t>
-        </is>
-      </c>
-      <c r="W3" s="5" t="n"/>
-      <c r="X3" s="5" t="n"/>
-      <c r="Y3" s="5" t="n"/>
-      <c r="Z3" s="3" t="n"/>
-      <c r="AA3" s="5" t="n"/>
-      <c r="AB3" s="4" t="inlineStr">
-        <is>
-          <t>道路附属物等</t>
-        </is>
-      </c>
-      <c r="AC3" s="5" t="n"/>
-      <c r="AD3" s="5" t="n"/>
-      <c r="AE3" s="5" t="n"/>
-      <c r="AF3" s="5" t="n"/>
-      <c r="AG3" s="6" t="n"/>
-    </row>
-    <row r="4" ht="17.01" customHeight="1">
-      <c r="F4" s="3" t="n"/>
-      <c r="G4" s="5" t="n"/>
-      <c r="H4" s="4" t="inlineStr">
-        <is>
-          <t>北海道</t>
-        </is>
-      </c>
-      <c r="I4" s="5" t="n"/>
-      <c r="J4" s="5" t="n"/>
-      <c r="K4" s="5" t="n"/>
-      <c r="L4" s="5" t="n"/>
-      <c r="M4" s="3" t="n"/>
-      <c r="N4" s="5" t="n"/>
-      <c r="O4" s="4" t="inlineStr">
-        <is>
-          <t>4,276</t>
-        </is>
-      </c>
-      <c r="P4" s="5" t="n"/>
-      <c r="Q4" s="5" t="n"/>
-      <c r="R4" s="5" t="n"/>
-      <c r="S4" s="3" t="n"/>
-      <c r="T4" s="5" t="n"/>
-      <c r="U4" s="5" t="n"/>
-      <c r="V4" s="5" t="n"/>
-      <c r="W4" s="4" t="inlineStr">
-        <is>
-          <t>273</t>
-        </is>
-      </c>
-      <c r="X4" s="5" t="n"/>
-      <c r="Y4" s="5" t="n"/>
-      <c r="Z4" s="3" t="n"/>
-      <c r="AA4" s="5" t="n"/>
-      <c r="AB4" s="5" t="n"/>
-      <c r="AC4" s="4" t="inlineStr">
-        <is>
-          <t>1,922</t>
-        </is>
-      </c>
-      <c r="AD4" s="5" t="n"/>
-      <c r="AE4" s="5" t="n"/>
-      <c r="AF4" s="5" t="n"/>
-      <c r="AG4" s="6" t="n"/>
     </row>
     <row r="5" ht="17.01" customHeight="1">
       <c r="F5" s="3" t="n"/>
-      <c r="G5" s="5" t="n"/>
-      <c r="H5" s="4" t="inlineStr">
-        <is>
-          <t>岩手県</t>
-        </is>
-      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>所在する都道府県</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="n"/>
       <c r="I5" s="5" t="n"/>
       <c r="J5" s="5" t="n"/>
       <c r="K5" s="5" t="n"/>
@@ -736,7 +749,7 @@
       <c r="N5" s="5" t="n"/>
       <c r="O5" s="4" t="inlineStr">
         <is>
-          <t>570</t>
+          <t>橋梁</t>
         </is>
       </c>
       <c r="P5" s="5" t="n"/>
@@ -745,22 +758,22 @@
       <c r="S5" s="8" t="n"/>
       <c r="T5" s="5" t="n"/>
       <c r="U5" s="5" t="n"/>
-      <c r="V5" s="5" t="n"/>
-      <c r="W5" s="4" t="inlineStr">
-        <is>
-          <t>71</t>
-        </is>
-      </c>
+      <c r="V5" s="4" t="inlineStr">
+        <is>
+          <t>トンネル</t>
+        </is>
+      </c>
+      <c r="W5" s="5" t="n"/>
       <c r="X5" s="5" t="n"/>
       <c r="Y5" s="5" t="n"/>
       <c r="Z5" s="8" t="n"/>
       <c r="AA5" s="5" t="n"/>
-      <c r="AB5" s="5" t="n"/>
-      <c r="AC5" s="4" t="inlineStr">
-        <is>
-          <t>190</t>
-        </is>
-      </c>
+      <c r="AB5" s="4" t="inlineStr">
+        <is>
+          <t>道路附属物等</t>
+        </is>
+      </c>
+      <c r="AC5" s="5" t="n"/>
       <c r="AD5" s="5" t="n"/>
       <c r="AE5" s="5" t="n"/>
       <c r="AF5" s="5" t="n"/>
@@ -771,7 +784,7 @@
       <c r="G6" s="10" t="n"/>
       <c r="H6" s="11" t="inlineStr">
         <is>
-          <t>宮城県</t>
+          <t>北海道</t>
         </is>
       </c>
       <c r="I6" s="10" t="n"/>
@@ -782,7 +795,7 @@
       <c r="N6" s="10" t="n"/>
       <c r="O6" s="11" t="inlineStr">
         <is>
-          <t>790</t>
+          <t>4,276</t>
         </is>
       </c>
       <c r="P6" s="10" t="n"/>
@@ -794,7 +807,7 @@
       <c r="V6" s="10" t="n"/>
       <c r="W6" s="11" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>273</t>
         </is>
       </c>
       <c r="X6" s="10" t="n"/>
@@ -804,7 +817,7 @@
       <c r="AB6" s="10" t="n"/>
       <c r="AC6" s="11" t="inlineStr">
         <is>
-          <t>177</t>
+          <t>1,922</t>
         </is>
       </c>
       <c r="AD6" s="10" t="n"/>
@@ -817,7 +830,7 @@
       <c r="G7" s="10" t="n"/>
       <c r="H7" s="11" t="inlineStr">
         <is>
-          <t>秋田県</t>
+          <t>青森県岩手県</t>
         </is>
       </c>
       <c r="I7" s="10" t="n"/>
@@ -828,7 +841,7 @@
       <c r="N7" s="10" t="n"/>
       <c r="O7" s="11" t="inlineStr">
         <is>
-          <t>689</t>
+          <t>319 570</t>
         </is>
       </c>
       <c r="P7" s="10" t="n"/>
@@ -840,7 +853,7 @@
       <c r="V7" s="10" t="n"/>
       <c r="W7" s="11" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>7 71</t>
         </is>
       </c>
       <c r="X7" s="10" t="n"/>
@@ -850,7 +863,7 @@
       <c r="AB7" s="10" t="n"/>
       <c r="AC7" s="11" t="inlineStr">
         <is>
-          <t>177</t>
+          <t>137 190</t>
         </is>
       </c>
       <c r="AD7" s="10" t="n"/>
@@ -863,7 +876,7 @@
       <c r="G8" s="10" t="n"/>
       <c r="H8" s="11" t="inlineStr">
         <is>
-          <t>山形県</t>
+          <t>宮城県</t>
         </is>
       </c>
       <c r="I8" s="10" t="n"/>
@@ -874,7 +887,7 @@
       <c r="N8" s="10" t="n"/>
       <c r="O8" s="11" t="inlineStr">
         <is>
-          <t>885</t>
+          <t>790</t>
         </is>
       </c>
       <c r="P8" s="10" t="n"/>
@@ -886,7 +899,7 @@
       <c r="V8" s="10" t="n"/>
       <c r="W8" s="11" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>27</t>
         </is>
       </c>
       <c r="X8" s="10" t="n"/>
@@ -896,7 +909,7 @@
       <c r="AB8" s="10" t="n"/>
       <c r="AC8" s="11" t="inlineStr">
         <is>
-          <t>199</t>
+          <t>177</t>
         </is>
       </c>
       <c r="AD8" s="10" t="n"/>
@@ -909,7 +922,7 @@
       <c r="G9" s="10" t="n"/>
       <c r="H9" s="11" t="inlineStr">
         <is>
-          <t>福島県</t>
+          <t>秋田県</t>
         </is>
       </c>
       <c r="I9" s="10" t="n"/>
@@ -920,7 +933,7 @@
       <c r="N9" s="10" t="n"/>
       <c r="O9" s="11" t="inlineStr">
         <is>
-          <t>873</t>
+          <t>689</t>
         </is>
       </c>
       <c r="P9" s="10" t="n"/>
@@ -932,7 +945,7 @@
       <c r="V9" s="10" t="n"/>
       <c r="W9" s="11" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>29</t>
         </is>
       </c>
       <c r="X9" s="10" t="n"/>
@@ -942,7 +955,7 @@
       <c r="AB9" s="10" t="n"/>
       <c r="AC9" s="11" t="inlineStr">
         <is>
-          <t>157</t>
+          <t>177</t>
         </is>
       </c>
       <c r="AD9" s="10" t="n"/>
@@ -955,7 +968,7 @@
       <c r="G10" s="10" t="n"/>
       <c r="H10" s="11" t="inlineStr">
         <is>
-          <t>茨城県</t>
+          <t>山形県</t>
         </is>
       </c>
       <c r="I10" s="10" t="n"/>
@@ -966,7 +979,7 @@
       <c r="N10" s="10" t="n"/>
       <c r="O10" s="11" t="inlineStr">
         <is>
-          <t>301</t>
+          <t>885</t>
         </is>
       </c>
       <c r="P10" s="10" t="n"/>
@@ -978,7 +991,7 @@
       <c r="V10" s="10" t="n"/>
       <c r="W10" s="11" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>45</t>
         </is>
       </c>
       <c r="X10" s="10" t="n"/>
@@ -988,7 +1001,7 @@
       <c r="AB10" s="10" t="n"/>
       <c r="AC10" s="11" t="inlineStr">
         <is>
-          <t>218</t>
+          <t>199</t>
         </is>
       </c>
       <c r="AD10" s="10" t="n"/>
@@ -1001,7 +1014,7 @@
       <c r="G11" s="10" t="n"/>
       <c r="H11" s="11" t="inlineStr">
         <is>
-          <t>群馬県</t>
+          <t>福島県</t>
         </is>
       </c>
       <c r="I11" s="10" t="n"/>
@@ -1012,7 +1025,7 @@
       <c r="N11" s="10" t="n"/>
       <c r="O11" s="11" t="inlineStr">
         <is>
-          <t>294</t>
+          <t>873</t>
         </is>
       </c>
       <c r="P11" s="10" t="n"/>
@@ -1024,7 +1037,7 @@
       <c r="V11" s="10" t="n"/>
       <c r="W11" s="11" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>51</t>
         </is>
       </c>
       <c r="X11" s="10" t="n"/>
@@ -1034,7 +1047,7 @@
       <c r="AB11" s="10" t="n"/>
       <c r="AC11" s="11" t="inlineStr">
         <is>
-          <t>135</t>
+          <t>157</t>
         </is>
       </c>
       <c r="AD11" s="10" t="n"/>
@@ -1047,7 +1060,7 @@
       <c r="G12" s="10" t="n"/>
       <c r="H12" s="11" t="inlineStr">
         <is>
-          <t>埼玉県</t>
+          <t>茨城県</t>
         </is>
       </c>
       <c r="I12" s="10" t="n"/>
@@ -1058,7 +1071,7 @@
       <c r="N12" s="10" t="n"/>
       <c r="O12" s="11" t="inlineStr">
         <is>
-          <t>545</t>
+          <t>301</t>
         </is>
       </c>
       <c r="P12" s="10" t="n"/>
@@ -1080,7 +1093,7 @@
       <c r="AB12" s="10" t="n"/>
       <c r="AC12" s="11" t="inlineStr">
         <is>
-          <t>417</t>
+          <t>218</t>
         </is>
       </c>
       <c r="AD12" s="10" t="n"/>
@@ -1093,7 +1106,7 @@
       <c r="G13" s="10" t="n"/>
       <c r="H13" s="11" t="inlineStr">
         <is>
-          <t>千葉県</t>
+          <t>栃木県群馬県</t>
         </is>
       </c>
       <c r="I13" s="10" t="n"/>
@@ -1104,7 +1117,7 @@
       <c r="N13" s="10" t="n"/>
       <c r="O13" s="11" t="inlineStr">
         <is>
-          <t>418</t>
+          <t>220 294</t>
         </is>
       </c>
       <c r="P13" s="10" t="n"/>
@@ -1116,7 +1129,7 @@
       <c r="V13" s="10" t="n"/>
       <c r="W13" s="11" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>0 3</t>
         </is>
       </c>
       <c r="X13" s="10" t="n"/>
@@ -1126,7 +1139,7 @@
       <c r="AB13" s="10" t="n"/>
       <c r="AC13" s="11" t="inlineStr">
         <is>
-          <t>253</t>
+          <t>149 135</t>
         </is>
       </c>
       <c r="AD13" s="10" t="n"/>
@@ -1139,7 +1152,7 @@
       <c r="G14" s="10" t="n"/>
       <c r="H14" s="11" t="inlineStr">
         <is>
-          <t>東京都</t>
+          <t>埼玉県</t>
         </is>
       </c>
       <c r="I14" s="10" t="n"/>
@@ -1150,7 +1163,7 @@
       <c r="N14" s="10" t="n"/>
       <c r="O14" s="11" t="inlineStr">
         <is>
-          <t>296</t>
+          <t>545</t>
         </is>
       </c>
       <c r="P14" s="10" t="n"/>
@@ -1162,7 +1175,7 @@
       <c r="V14" s="10" t="n"/>
       <c r="W14" s="11" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="X14" s="10" t="n"/>
@@ -1172,7 +1185,7 @@
       <c r="AB14" s="10" t="n"/>
       <c r="AC14" s="11" t="inlineStr">
         <is>
-          <t>485</t>
+          <t>417</t>
         </is>
       </c>
       <c r="AD14" s="10" t="n"/>
@@ -1185,7 +1198,7 @@
       <c r="G15" s="10" t="n"/>
       <c r="H15" s="11" t="inlineStr">
         <is>
-          <t>神奈川県</t>
+          <t>千葉県</t>
         </is>
       </c>
       <c r="I15" s="10" t="n"/>
@@ -1196,7 +1209,7 @@
       <c r="N15" s="10" t="n"/>
       <c r="O15" s="11" t="inlineStr">
         <is>
-          <t>409</t>
+          <t>418</t>
         </is>
       </c>
       <c r="P15" s="10" t="n"/>
@@ -1218,7 +1231,7 @@
       <c r="AB15" s="10" t="n"/>
       <c r="AC15" s="11" t="inlineStr">
         <is>
-          <t>316</t>
+          <t>253</t>
         </is>
       </c>
       <c r="AD15" s="10" t="n"/>
@@ -1231,7 +1244,7 @@
       <c r="G16" s="10" t="n"/>
       <c r="H16" s="11" t="inlineStr">
         <is>
-          <t>新潟県</t>
+          <t>東京都</t>
         </is>
       </c>
       <c r="I16" s="10" t="n"/>
@@ -1242,7 +1255,7 @@
       <c r="N16" s="10" t="n"/>
       <c r="O16" s="11" t="inlineStr">
         <is>
-          <t>1,663</t>
+          <t>296</t>
         </is>
       </c>
       <c r="P16" s="10" t="n"/>
@@ -1254,7 +1267,7 @@
       <c r="V16" s="10" t="n"/>
       <c r="W16" s="11" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>3</t>
         </is>
       </c>
       <c r="X16" s="10" t="n"/>
@@ -1264,7 +1277,7 @@
       <c r="AB16" s="10" t="n"/>
       <c r="AC16" s="11" t="inlineStr">
         <is>
-          <t>414</t>
+          <t>485</t>
         </is>
       </c>
       <c r="AD16" s="10" t="n"/>
@@ -1277,7 +1290,7 @@
       <c r="G17" s="10" t="n"/>
       <c r="H17" s="11" t="inlineStr">
         <is>
-          <t>石川県</t>
+          <t>神奈川県</t>
         </is>
       </c>
       <c r="I17" s="10" t="n"/>
@@ -1288,7 +1301,7 @@
       <c r="N17" s="10" t="n"/>
       <c r="O17" s="11" t="inlineStr">
         <is>
-          <t>880</t>
+          <t>409</t>
         </is>
       </c>
       <c r="P17" s="10" t="n"/>
@@ -1300,7 +1313,7 @@
       <c r="V17" s="10" t="n"/>
       <c r="W17" s="11" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>26</t>
         </is>
       </c>
       <c r="X17" s="10" t="n"/>
@@ -1310,7 +1323,7 @@
       <c r="AB17" s="10" t="n"/>
       <c r="AC17" s="11" t="inlineStr">
         <is>
-          <t>139</t>
+          <t>316</t>
         </is>
       </c>
       <c r="AD17" s="10" t="n"/>
@@ -1323,7 +1336,7 @@
       <c r="G18" s="10" t="n"/>
       <c r="H18" s="11" t="inlineStr">
         <is>
-          <t>福井県</t>
+          <t>新潟県</t>
         </is>
       </c>
       <c r="I18" s="10" t="n"/>
@@ -1334,7 +1347,7 @@
       <c r="N18" s="10" t="n"/>
       <c r="O18" s="11" t="inlineStr">
         <is>
-          <t>487</t>
+          <t>1,663</t>
         </is>
       </c>
       <c r="P18" s="10" t="n"/>
@@ -1346,7 +1359,7 @@
       <c r="V18" s="10" t="n"/>
       <c r="W18" s="11" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>47</t>
         </is>
       </c>
       <c r="X18" s="10" t="n"/>
@@ -1354,12 +1367,12 @@
       <c r="Z18" s="12" t="n"/>
       <c r="AA18" s="10" t="n"/>
       <c r="AB18" s="10" t="n"/>
-      <c r="AC18" s="10" t="n"/>
-      <c r="AD18" s="11" t="inlineStr">
-        <is>
-          <t>71</t>
-        </is>
-      </c>
+      <c r="AC18" s="11" t="inlineStr">
+        <is>
+          <t>414</t>
+        </is>
+      </c>
+      <c r="AD18" s="10" t="n"/>
       <c r="AE18" s="10" t="n"/>
       <c r="AF18" s="10" t="n"/>
       <c r="AG18" s="13" t="n"/>
@@ -1369,7 +1382,7 @@
       <c r="G19" s="10" t="n"/>
       <c r="H19" s="11" t="inlineStr">
         <is>
-          <t>山梨県</t>
+          <t>富山県石川県</t>
         </is>
       </c>
       <c r="I19" s="10" t="n"/>
@@ -1380,7 +1393,7 @@
       <c r="N19" s="10" t="n"/>
       <c r="O19" s="11" t="inlineStr">
         <is>
-          <t>342</t>
+          <t>912 880</t>
         </is>
       </c>
       <c r="P19" s="10" t="n"/>
@@ -1392,7 +1405,7 @@
       <c r="V19" s="10" t="n"/>
       <c r="W19" s="11" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>29 18</t>
         </is>
       </c>
       <c r="X19" s="10" t="n"/>
@@ -1400,12 +1413,12 @@
       <c r="Z19" s="12" t="n"/>
       <c r="AA19" s="10" t="n"/>
       <c r="AB19" s="10" t="n"/>
-      <c r="AC19" s="10" t="n"/>
-      <c r="AD19" s="11" t="inlineStr">
-        <is>
-          <t>94</t>
-        </is>
-      </c>
+      <c r="AC19" s="11" t="inlineStr">
+        <is>
+          <t>120 139</t>
+        </is>
+      </c>
+      <c r="AD19" s="10" t="n"/>
       <c r="AE19" s="10" t="n"/>
       <c r="AF19" s="10" t="n"/>
       <c r="AG19" s="13" t="n"/>
@@ -1415,7 +1428,7 @@
       <c r="G20" s="10" t="n"/>
       <c r="H20" s="11" t="inlineStr">
         <is>
-          <t>長野県</t>
+          <t>福井県</t>
         </is>
       </c>
       <c r="I20" s="10" t="n"/>
@@ -1426,7 +1439,7 @@
       <c r="N20" s="10" t="n"/>
       <c r="O20" s="11" t="inlineStr">
         <is>
-          <t>818</t>
+          <t>487</t>
         </is>
       </c>
       <c r="P20" s="10" t="n"/>
@@ -1438,7 +1451,7 @@
       <c r="V20" s="10" t="n"/>
       <c r="W20" s="11" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>32</t>
         </is>
       </c>
       <c r="X20" s="10" t="n"/>
@@ -1446,12 +1459,12 @@
       <c r="Z20" s="12" t="n"/>
       <c r="AA20" s="10" t="n"/>
       <c r="AB20" s="10" t="n"/>
-      <c r="AC20" s="11" t="inlineStr">
-        <is>
-          <t>229</t>
-        </is>
-      </c>
-      <c r="AD20" s="10" t="n"/>
+      <c r="AC20" s="10" t="n"/>
+      <c r="AD20" s="11" t="inlineStr">
+        <is>
+          <t>71</t>
+        </is>
+      </c>
       <c r="AE20" s="10" t="n"/>
       <c r="AF20" s="10" t="n"/>
       <c r="AG20" s="13" t="n"/>
@@ -1461,7 +1474,7 @@
       <c r="G21" s="10" t="n"/>
       <c r="H21" s="11" t="inlineStr">
         <is>
-          <t>岐阜県</t>
+          <t>山梨県</t>
         </is>
       </c>
       <c r="I21" s="10" t="n"/>
@@ -1472,7 +1485,7 @@
       <c r="N21" s="10" t="n"/>
       <c r="O21" s="11" t="inlineStr">
         <is>
-          <t>1,070</t>
+          <t>342</t>
         </is>
       </c>
       <c r="P21" s="10" t="n"/>
@@ -1484,7 +1497,7 @@
       <c r="V21" s="10" t="n"/>
       <c r="W21" s="11" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>13</t>
         </is>
       </c>
       <c r="X21" s="10" t="n"/>
@@ -1492,12 +1505,12 @@
       <c r="Z21" s="12" t="n"/>
       <c r="AA21" s="10" t="n"/>
       <c r="AB21" s="10" t="n"/>
-      <c r="AC21" s="11" t="inlineStr">
-        <is>
-          <t>481</t>
-        </is>
-      </c>
-      <c r="AD21" s="10" t="n"/>
+      <c r="AC21" s="10" t="n"/>
+      <c r="AD21" s="11" t="inlineStr">
+        <is>
+          <t>94</t>
+        </is>
+      </c>
       <c r="AE21" s="10" t="n"/>
       <c r="AF21" s="10" t="n"/>
       <c r="AG21" s="13" t="n"/>
@@ -1507,7 +1520,7 @@
       <c r="G22" s="10" t="n"/>
       <c r="H22" s="11" t="inlineStr">
         <is>
-          <t>静岡県</t>
+          <t>長野県</t>
         </is>
       </c>
       <c r="I22" s="10" t="n"/>
@@ -1518,7 +1531,7 @@
       <c r="N22" s="10" t="n"/>
       <c r="O22" s="11" t="inlineStr">
         <is>
-          <t>1,176</t>
+          <t>818</t>
         </is>
       </c>
       <c r="P22" s="10" t="n"/>
@@ -1540,7 +1553,7 @@
       <c r="AB22" s="10" t="n"/>
       <c r="AC22" s="11" t="inlineStr">
         <is>
-          <t>329</t>
+          <t>229</t>
         </is>
       </c>
       <c r="AD22" s="10" t="n"/>
@@ -1553,7 +1566,7 @@
       <c r="G23" s="10" t="n"/>
       <c r="H23" s="11" t="inlineStr">
         <is>
-          <t>三重県</t>
+          <t>岐阜県</t>
         </is>
       </c>
       <c r="I23" s="10" t="n"/>
@@ -1564,7 +1577,7 @@
       <c r="N23" s="10" t="n"/>
       <c r="O23" s="11" t="inlineStr">
         <is>
-          <t>1,461</t>
+          <t>1,070</t>
         </is>
       </c>
       <c r="P23" s="10" t="n"/>
@@ -1576,7 +1589,7 @@
       <c r="V23" s="10" t="n"/>
       <c r="W23" s="11" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>36</t>
         </is>
       </c>
       <c r="X23" s="10" t="n"/>
@@ -1586,7 +1599,7 @@
       <c r="AB23" s="10" t="n"/>
       <c r="AC23" s="11" t="inlineStr">
         <is>
-          <t>287</t>
+          <t>481</t>
         </is>
       </c>
       <c r="AD23" s="10" t="n"/>
@@ -1599,7 +1612,7 @@
       <c r="G24" s="10" t="n"/>
       <c r="H24" s="11" t="inlineStr">
         <is>
-          <t>滋賀県</t>
+          <t>静岡県</t>
         </is>
       </c>
       <c r="I24" s="10" t="n"/>
@@ -1610,7 +1623,7 @@
       <c r="N24" s="10" t="n"/>
       <c r="O24" s="11" t="inlineStr">
         <is>
-          <t>800</t>
+          <t>1,176</t>
         </is>
       </c>
       <c r="P24" s="10" t="n"/>
@@ -1622,7 +1635,7 @@
       <c r="V24" s="10" t="n"/>
       <c r="W24" s="11" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>28</t>
         </is>
       </c>
       <c r="X24" s="10" t="n"/>
@@ -1630,12 +1643,12 @@
       <c r="Z24" s="12" t="n"/>
       <c r="AA24" s="10" t="n"/>
       <c r="AB24" s="10" t="n"/>
-      <c r="AC24" s="10" t="n"/>
-      <c r="AD24" s="11" t="inlineStr">
-        <is>
-          <t>99</t>
-        </is>
-      </c>
+      <c r="AC24" s="11" t="inlineStr">
+        <is>
+          <t>329</t>
+        </is>
+      </c>
+      <c r="AD24" s="10" t="n"/>
       <c r="AE24" s="10" t="n"/>
       <c r="AF24" s="10" t="n"/>
       <c r="AG24" s="13" t="n"/>
@@ -1645,7 +1658,7 @@
       <c r="G25" s="10" t="n"/>
       <c r="H25" s="11" t="inlineStr">
         <is>
-          <t>京都府</t>
+          <t>愛知県三重県</t>
         </is>
       </c>
       <c r="I25" s="10" t="n"/>
@@ -1656,7 +1669,7 @@
       <c r="N25" s="10" t="n"/>
       <c r="O25" s="11" t="inlineStr">
         <is>
-          <t>699</t>
+          <t>1,460 1,461</t>
         </is>
       </c>
       <c r="P25" s="10" t="n"/>
@@ -1668,7 +1681,7 @@
       <c r="V25" s="10" t="n"/>
       <c r="W25" s="11" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>13 38</t>
         </is>
       </c>
       <c r="X25" s="10" t="n"/>
@@ -1678,7 +1691,7 @@
       <c r="AB25" s="10" t="n"/>
       <c r="AC25" s="11" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>706 287</t>
         </is>
       </c>
       <c r="AD25" s="10" t="n"/>
@@ -1691,7 +1704,7 @@
       <c r="G26" s="10" t="n"/>
       <c r="H26" s="11" t="inlineStr">
         <is>
-          <t>大阪府</t>
+          <t>滋賀県</t>
         </is>
       </c>
       <c r="I26" s="10" t="n"/>
@@ -1702,7 +1715,7 @@
       <c r="N26" s="10" t="n"/>
       <c r="O26" s="11" t="inlineStr">
         <is>
-          <t>460</t>
+          <t>800</t>
         </is>
       </c>
       <c r="P26" s="10" t="n"/>
@@ -1714,7 +1727,7 @@
       <c r="V26" s="10" t="n"/>
       <c r="W26" s="11" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>10</t>
         </is>
       </c>
       <c r="X26" s="10" t="n"/>
@@ -1722,12 +1735,12 @@
       <c r="Z26" s="12" t="n"/>
       <c r="AA26" s="10" t="n"/>
       <c r="AB26" s="10" t="n"/>
-      <c r="AC26" s="11" t="inlineStr">
-        <is>
-          <t>480</t>
-        </is>
-      </c>
-      <c r="AD26" s="10" t="n"/>
+      <c r="AC26" s="10" t="n"/>
+      <c r="AD26" s="11" t="inlineStr">
+        <is>
+          <t>99</t>
+        </is>
+      </c>
       <c r="AE26" s="10" t="n"/>
       <c r="AF26" s="10" t="n"/>
       <c r="AG26" s="13" t="n"/>
@@ -1737,7 +1750,7 @@
       <c r="G27" s="10" t="n"/>
       <c r="H27" s="11" t="inlineStr">
         <is>
-          <t>兵庫県</t>
+          <t>京都府</t>
         </is>
       </c>
       <c r="I27" s="10" t="n"/>
@@ -1748,7 +1761,7 @@
       <c r="N27" s="10" t="n"/>
       <c r="O27" s="11" t="inlineStr">
         <is>
-          <t>1,254</t>
+          <t>699</t>
         </is>
       </c>
       <c r="P27" s="10" t="n"/>
@@ -1760,7 +1773,7 @@
       <c r="V27" s="10" t="n"/>
       <c r="W27" s="11" t="inlineStr">
         <is>
-          <t>58</t>
+          <t>10</t>
         </is>
       </c>
       <c r="X27" s="10" t="n"/>
@@ -1770,7 +1783,7 @@
       <c r="AB27" s="10" t="n"/>
       <c r="AC27" s="11" t="inlineStr">
         <is>
-          <t>439</t>
+          <t>180</t>
         </is>
       </c>
       <c r="AD27" s="10" t="n"/>
@@ -1783,7 +1796,7 @@
       <c r="G28" s="10" t="n"/>
       <c r="H28" s="11" t="inlineStr">
         <is>
-          <t>奈良県</t>
+          <t>大阪府</t>
         </is>
       </c>
       <c r="I28" s="10" t="n"/>
@@ -1794,7 +1807,7 @@
       <c r="N28" s="10" t="n"/>
       <c r="O28" s="11" t="inlineStr">
         <is>
-          <t>463</t>
+          <t>460</t>
         </is>
       </c>
       <c r="P28" s="10" t="n"/>
@@ -1806,7 +1819,7 @@
       <c r="V28" s="10" t="n"/>
       <c r="W28" s="11" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>16</t>
         </is>
       </c>
       <c r="X28" s="10" t="n"/>
@@ -1816,7 +1829,7 @@
       <c r="AB28" s="10" t="n"/>
       <c r="AC28" s="11" t="inlineStr">
         <is>
-          <t>137</t>
+          <t>480</t>
         </is>
       </c>
       <c r="AD28" s="10" t="n"/>
@@ -1829,7 +1842,7 @@
       <c r="G29" s="10" t="n"/>
       <c r="H29" s="11" t="inlineStr">
         <is>
-          <t>鳥取県</t>
+          <t>兵庫県</t>
         </is>
       </c>
       <c r="I29" s="10" t="n"/>
@@ -1840,7 +1853,7 @@
       <c r="N29" s="10" t="n"/>
       <c r="O29" s="11" t="inlineStr">
         <is>
-          <t>761</t>
+          <t>1,254</t>
         </is>
       </c>
       <c r="P29" s="10" t="n"/>
@@ -1852,7 +1865,7 @@
       <c r="V29" s="10" t="n"/>
       <c r="W29" s="11" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>58</t>
         </is>
       </c>
       <c r="X29" s="10" t="n"/>
@@ -1862,14 +1875,10 @@
       <c r="AB29" s="10" t="n"/>
       <c r="AC29" s="11" t="inlineStr">
         <is>
-          <t>144</t>
-        </is>
-      </c>
-      <c r="AD29" s="11" t="inlineStr">
-        <is>
-          <t>92</t>
-        </is>
-      </c>
+          <t>439</t>
+        </is>
+      </c>
+      <c r="AD29" s="10" t="n"/>
       <c r="AE29" s="10" t="n"/>
       <c r="AF29" s="10" t="n"/>
       <c r="AG29" s="13" t="n"/>
@@ -1879,7 +1888,7 @@
       <c r="G30" s="10" t="n"/>
       <c r="H30" s="11" t="inlineStr">
         <is>
-          <t>島根県</t>
+          <t>奈良県</t>
         </is>
       </c>
       <c r="I30" s="10" t="n"/>
@@ -1890,7 +1899,7 @@
       <c r="N30" s="10" t="n"/>
       <c r="O30" s="11" t="inlineStr">
         <is>
-          <t>707</t>
+          <t>463</t>
         </is>
       </c>
       <c r="P30" s="10" t="n"/>
@@ -1902,7 +1911,7 @@
       <c r="V30" s="10" t="n"/>
       <c r="W30" s="11" t="inlineStr">
         <is>
-          <t>52</t>
+          <t>7</t>
         </is>
       </c>
       <c r="X30" s="10" t="n"/>
@@ -1912,7 +1921,7 @@
       <c r="AB30" s="10" t="n"/>
       <c r="AC30" s="11" t="inlineStr">
         <is>
-          <t>165</t>
+          <t>137</t>
         </is>
       </c>
       <c r="AD30" s="10" t="n"/>
@@ -1925,7 +1934,7 @@
       <c r="G31" s="10" t="n"/>
       <c r="H31" s="11" t="inlineStr">
         <is>
-          <t>岡山県</t>
+          <t>和歌山県鳥取県</t>
         </is>
       </c>
       <c r="I31" s="10" t="n"/>
@@ -1936,7 +1945,7 @@
       <c r="N31" s="10" t="n"/>
       <c r="O31" s="11" t="inlineStr">
         <is>
-          <t>1,065</t>
+          <t>701 761</t>
         </is>
       </c>
       <c r="P31" s="10" t="n"/>
@@ -1948,7 +1957,7 @@
       <c r="V31" s="10" t="n"/>
       <c r="W31" s="11" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>80 39</t>
         </is>
       </c>
       <c r="X31" s="10" t="n"/>
@@ -1958,10 +1967,14 @@
       <c r="AB31" s="10" t="n"/>
       <c r="AC31" s="11" t="inlineStr">
         <is>
-          <t>172</t>
-        </is>
-      </c>
-      <c r="AD31" s="10" t="n"/>
+          <t>144</t>
+        </is>
+      </c>
+      <c r="AD31" s="11" t="inlineStr">
+        <is>
+          <t>92</t>
+        </is>
+      </c>
       <c r="AE31" s="10" t="n"/>
       <c r="AF31" s="10" t="n"/>
       <c r="AG31" s="13" t="n"/>
@@ -1971,7 +1984,7 @@
       <c r="G32" s="10" t="n"/>
       <c r="H32" s="11" t="inlineStr">
         <is>
-          <t>広島県</t>
+          <t>島根県</t>
         </is>
       </c>
       <c r="I32" s="10" t="n"/>
@@ -1982,7 +1995,7 @@
       <c r="N32" s="10" t="n"/>
       <c r="O32" s="11" t="inlineStr">
         <is>
-          <t>995</t>
+          <t>707</t>
         </is>
       </c>
       <c r="P32" s="10" t="n"/>
@@ -1994,7 +2007,7 @@
       <c r="V32" s="10" t="n"/>
       <c r="W32" s="11" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>52</t>
         </is>
       </c>
       <c r="X32" s="10" t="n"/>
@@ -2004,7 +2017,7 @@
       <c r="AB32" s="10" t="n"/>
       <c r="AC32" s="11" t="inlineStr">
         <is>
-          <t>262</t>
+          <t>165</t>
         </is>
       </c>
       <c r="AD32" s="10" t="n"/>
@@ -2017,7 +2030,7 @@
       <c r="G33" s="10" t="n"/>
       <c r="H33" s="11" t="inlineStr">
         <is>
-          <t>山口県</t>
+          <t>岡山県</t>
         </is>
       </c>
       <c r="I33" s="10" t="n"/>
@@ -2028,7 +2041,7 @@
       <c r="N33" s="10" t="n"/>
       <c r="O33" s="11" t="inlineStr">
         <is>
-          <t>1,351</t>
+          <t>1,065</t>
         </is>
       </c>
       <c r="P33" s="10" t="n"/>
@@ -2040,7 +2053,7 @@
       <c r="V33" s="10" t="n"/>
       <c r="W33" s="11" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>21</t>
         </is>
       </c>
       <c r="X33" s="10" t="n"/>
@@ -2050,7 +2063,7 @@
       <c r="AB33" s="10" t="n"/>
       <c r="AC33" s="11" t="inlineStr">
         <is>
-          <t>196</t>
+          <t>172</t>
         </is>
       </c>
       <c r="AD33" s="10" t="n"/>
@@ -2063,7 +2076,7 @@
       <c r="G34" s="10" t="n"/>
       <c r="H34" s="11" t="inlineStr">
         <is>
-          <t>徳島県</t>
+          <t>広島県</t>
         </is>
       </c>
       <c r="I34" s="10" t="n"/>
@@ -2074,7 +2087,7 @@
       <c r="N34" s="10" t="n"/>
       <c r="O34" s="11" t="inlineStr">
         <is>
-          <t>442</t>
+          <t>995</t>
         </is>
       </c>
       <c r="P34" s="10" t="n"/>
@@ -2086,7 +2099,7 @@
       <c r="V34" s="10" t="n"/>
       <c r="W34" s="11" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>90</t>
         </is>
       </c>
       <c r="X34" s="10" t="n"/>
@@ -2096,7 +2109,7 @@
       <c r="AB34" s="10" t="n"/>
       <c r="AC34" s="11" t="inlineStr">
         <is>
-          <t>153</t>
+          <t>262</t>
         </is>
       </c>
       <c r="AD34" s="10" t="n"/>
@@ -2109,7 +2122,7 @@
       <c r="G35" s="10" t="n"/>
       <c r="H35" s="11" t="inlineStr">
         <is>
-          <t>愛媛県</t>
+          <t>山口県</t>
         </is>
       </c>
       <c r="I35" s="10" t="n"/>
@@ -2120,7 +2133,7 @@
       <c r="N35" s="10" t="n"/>
       <c r="O35" s="11" t="inlineStr">
         <is>
-          <t>906</t>
+          <t>1,351</t>
         </is>
       </c>
       <c r="P35" s="10" t="n"/>
@@ -2132,7 +2145,7 @@
       <c r="V35" s="10" t="n"/>
       <c r="W35" s="11" t="inlineStr">
         <is>
-          <t>56</t>
+          <t>40</t>
         </is>
       </c>
       <c r="X35" s="10" t="n"/>
@@ -2142,7 +2155,7 @@
       <c r="AB35" s="10" t="n"/>
       <c r="AC35" s="11" t="inlineStr">
         <is>
-          <t>255</t>
+          <t>196</t>
         </is>
       </c>
       <c r="AD35" s="10" t="n"/>
@@ -2155,7 +2168,7 @@
       <c r="G36" s="10" t="n"/>
       <c r="H36" s="11" t="inlineStr">
         <is>
-          <t>高知県</t>
+          <t>徳島県</t>
         </is>
       </c>
       <c r="I36" s="10" t="n"/>
@@ -2166,7 +2179,7 @@
       <c r="N36" s="10" t="n"/>
       <c r="O36" s="11" t="inlineStr">
         <is>
-          <t>853</t>
+          <t>442</t>
         </is>
       </c>
       <c r="P36" s="10" t="n"/>
@@ -2178,7 +2191,7 @@
       <c r="V36" s="10" t="n"/>
       <c r="W36" s="11" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>33</t>
         </is>
       </c>
       <c r="X36" s="10" t="n"/>
@@ -2188,7 +2201,7 @@
       <c r="AB36" s="10" t="n"/>
       <c r="AC36" s="11" t="inlineStr">
         <is>
-          <t>199</t>
+          <t>153</t>
         </is>
       </c>
       <c r="AD36" s="10" t="n"/>
@@ -2201,7 +2214,7 @@
       <c r="G37" s="10" t="n"/>
       <c r="H37" s="11" t="inlineStr">
         <is>
-          <t>福岡県</t>
+          <t>香川県愛媛県</t>
         </is>
       </c>
       <c r="I37" s="10" t="n"/>
@@ -2212,7 +2225,7 @@
       <c r="N37" s="10" t="n"/>
       <c r="O37" s="11" t="inlineStr">
         <is>
-          <t>1,299</t>
+          <t>471 906</t>
         </is>
       </c>
       <c r="P37" s="10" t="n"/>
@@ -2224,7 +2237,7 @@
       <c r="V37" s="10" t="n"/>
       <c r="W37" s="11" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>9 56</t>
         </is>
       </c>
       <c r="X37" s="10" t="n"/>
@@ -2234,7 +2247,7 @@
       <c r="AB37" s="10" t="n"/>
       <c r="AC37" s="11" t="inlineStr">
         <is>
-          <t>181</t>
+          <t>186 255</t>
         </is>
       </c>
       <c r="AD37" s="10" t="n"/>
@@ -2247,7 +2260,7 @@
       <c r="G38" s="10" t="n"/>
       <c r="H38" s="11" t="inlineStr">
         <is>
-          <t>佐賀県</t>
+          <t>高知県</t>
         </is>
       </c>
       <c r="I38" s="10" t="n"/>
@@ -2258,7 +2271,7 @@
       <c r="N38" s="10" t="n"/>
       <c r="O38" s="11" t="inlineStr">
         <is>
-          <t>783</t>
+          <t>853</t>
         </is>
       </c>
       <c r="P38" s="10" t="n"/>
@@ -2270,7 +2283,7 @@
       <c r="V38" s="10" t="n"/>
       <c r="W38" s="11" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>70</t>
         </is>
       </c>
       <c r="X38" s="10" t="n"/>
@@ -2278,12 +2291,12 @@
       <c r="Z38" s="12" t="n"/>
       <c r="AA38" s="10" t="n"/>
       <c r="AB38" s="10" t="n"/>
-      <c r="AC38" s="10" t="n"/>
-      <c r="AD38" s="11" t="inlineStr">
-        <is>
-          <t>88</t>
-        </is>
-      </c>
+      <c r="AC38" s="11" t="inlineStr">
+        <is>
+          <t>199</t>
+        </is>
+      </c>
+      <c r="AD38" s="10" t="n"/>
       <c r="AE38" s="10" t="n"/>
       <c r="AF38" s="10" t="n"/>
       <c r="AG38" s="13" t="n"/>
@@ -2293,7 +2306,7 @@
       <c r="G39" s="10" t="n"/>
       <c r="H39" s="11" t="inlineStr">
         <is>
-          <t>長崎県</t>
+          <t>福岡県</t>
         </is>
       </c>
       <c r="I39" s="10" t="n"/>
@@ -2304,7 +2317,7 @@
       <c r="N39" s="10" t="n"/>
       <c r="O39" s="11" t="inlineStr">
         <is>
-          <t>249</t>
+          <t>1,299</t>
         </is>
       </c>
       <c r="P39" s="10" t="n"/>
@@ -2316,7 +2329,7 @@
       <c r="V39" s="10" t="n"/>
       <c r="W39" s="11" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>15</t>
         </is>
       </c>
       <c r="X39" s="10" t="n"/>
@@ -2324,12 +2337,12 @@
       <c r="Z39" s="12" t="n"/>
       <c r="AA39" s="10" t="n"/>
       <c r="AB39" s="10" t="n"/>
-      <c r="AC39" s="10" t="n"/>
-      <c r="AD39" s="11" t="inlineStr">
-        <is>
-          <t>66</t>
-        </is>
-      </c>
+      <c r="AC39" s="11" t="inlineStr">
+        <is>
+          <t>181</t>
+        </is>
+      </c>
+      <c r="AD39" s="10" t="n"/>
       <c r="AE39" s="10" t="n"/>
       <c r="AF39" s="10" t="n"/>
       <c r="AG39" s="13" t="n"/>
@@ -2339,7 +2352,7 @@
       <c r="G40" s="10" t="n"/>
       <c r="H40" s="11" t="inlineStr">
         <is>
-          <t>大分県</t>
+          <t>佐賀県</t>
         </is>
       </c>
       <c r="I40" s="10" t="n"/>
@@ -2350,7 +2363,7 @@
       <c r="N40" s="10" t="n"/>
       <c r="O40" s="11" t="inlineStr">
         <is>
-          <t>543</t>
+          <t>783</t>
         </is>
       </c>
       <c r="P40" s="10" t="n"/>
@@ -2362,7 +2375,7 @@
       <c r="V40" s="10" t="n"/>
       <c r="W40" s="11" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>12</t>
         </is>
       </c>
       <c r="X40" s="10" t="n"/>
@@ -2370,12 +2383,12 @@
       <c r="Z40" s="12" t="n"/>
       <c r="AA40" s="10" t="n"/>
       <c r="AB40" s="10" t="n"/>
-      <c r="AC40" s="11" t="inlineStr">
-        <is>
-          <t>110</t>
-        </is>
-      </c>
-      <c r="AD40" s="10" t="n"/>
+      <c r="AC40" s="10" t="n"/>
+      <c r="AD40" s="11" t="inlineStr">
+        <is>
+          <t>88</t>
+        </is>
+      </c>
       <c r="AE40" s="10" t="n"/>
       <c r="AF40" s="10" t="n"/>
       <c r="AG40" s="13" t="n"/>
@@ -2385,7 +2398,7 @@
       <c r="G41" s="10" t="n"/>
       <c r="H41" s="11" t="inlineStr">
         <is>
-          <t>宮崎県</t>
+          <t>長崎県</t>
         </is>
       </c>
       <c r="I41" s="10" t="n"/>
@@ -2396,7 +2409,7 @@
       <c r="N41" s="10" t="n"/>
       <c r="O41" s="11" t="inlineStr">
         <is>
-          <t>540</t>
+          <t>249</t>
         </is>
       </c>
       <c r="P41" s="10" t="n"/>
@@ -2408,7 +2421,7 @@
       <c r="V41" s="10" t="n"/>
       <c r="W41" s="11" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>8</t>
         </is>
       </c>
       <c r="X41" s="10" t="n"/>
@@ -2416,12 +2429,12 @@
       <c r="Z41" s="12" t="n"/>
       <c r="AA41" s="10" t="n"/>
       <c r="AB41" s="10" t="n"/>
-      <c r="AC41" s="11" t="inlineStr">
-        <is>
-          <t>153</t>
-        </is>
-      </c>
-      <c r="AD41" s="10" t="n"/>
+      <c r="AC41" s="10" t="n"/>
+      <c r="AD41" s="11" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
       <c r="AE41" s="10" t="n"/>
       <c r="AF41" s="10" t="n"/>
       <c r="AG41" s="13" t="n"/>
@@ -2431,7 +2444,7 @@
       <c r="G42" s="10" t="n"/>
       <c r="H42" s="11" t="inlineStr">
         <is>
-          <t>鹿児島県</t>
+          <t>熊本県大分県</t>
         </is>
       </c>
       <c r="I42" s="10" t="n"/>
@@ -2442,7 +2455,7 @@
       <c r="N42" s="10" t="n"/>
       <c r="O42" s="11" t="inlineStr">
         <is>
-          <t>552</t>
+          <t>546 543</t>
         </is>
       </c>
       <c r="P42" s="10" t="n"/>
@@ -2454,7 +2467,7 @@
       <c r="V42" s="10" t="n"/>
       <c r="W42" s="11" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>15 48</t>
         </is>
       </c>
       <c r="X42" s="10" t="n"/>
@@ -2464,7 +2477,7 @@
       <c r="AB42" s="10" t="n"/>
       <c r="AC42" s="11" t="inlineStr">
         <is>
-          <t>108</t>
+          <t>151 110</t>
         </is>
       </c>
       <c r="AD42" s="10" t="n"/>
@@ -2477,7 +2490,7 @@
       <c r="G43" s="10" t="n"/>
       <c r="H43" s="11" t="inlineStr">
         <is>
-          <t>沖縄県</t>
+          <t>宮崎県</t>
         </is>
       </c>
       <c r="I43" s="10" t="n"/>
@@ -2488,7 +2501,7 @@
       <c r="N43" s="10" t="n"/>
       <c r="O43" s="11" t="inlineStr">
         <is>
-          <t>398</t>
+          <t>540</t>
         </is>
       </c>
       <c r="P43" s="10" t="n"/>
@@ -2500,7 +2513,7 @@
       <c r="V43" s="10" t="n"/>
       <c r="W43" s="11" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>44</t>
         </is>
       </c>
       <c r="X43" s="10" t="n"/>
@@ -2510,7 +2523,7 @@
       <c r="AB43" s="10" t="n"/>
       <c r="AC43" s="11" t="inlineStr">
         <is>
-          <t>127</t>
+          <t>153</t>
         </is>
       </c>
       <c r="AD43" s="10" t="n"/>
@@ -2521,12 +2534,12 @@
     <row r="44" ht="17.01" customHeight="1">
       <c r="F44" s="9" t="n"/>
       <c r="G44" s="10" t="n"/>
-      <c r="H44" s="10" t="n"/>
-      <c r="I44" s="11" t="inlineStr">
-        <is>
-          <t>合計</t>
-        </is>
-      </c>
+      <c r="H44" s="11" t="inlineStr">
+        <is>
+          <t>鹿児島県</t>
+        </is>
+      </c>
+      <c r="I44" s="10" t="n"/>
       <c r="J44" s="10" t="n"/>
       <c r="K44" s="10" t="n"/>
       <c r="L44" s="10" t="n"/>
@@ -2534,7 +2547,7 @@
       <c r="N44" s="10" t="n"/>
       <c r="O44" s="11" t="inlineStr">
         <is>
-          <t>37,992</t>
+          <t>552</t>
         </is>
       </c>
       <c r="P44" s="10" t="n"/>
@@ -2543,12 +2556,12 @@
       <c r="S44" s="12" t="n"/>
       <c r="T44" s="10" t="n"/>
       <c r="U44" s="10" t="n"/>
-      <c r="V44" s="11" t="inlineStr">
-        <is>
-          <t>1,610</t>
-        </is>
-      </c>
-      <c r="W44" s="10" t="n"/>
+      <c r="V44" s="10" t="n"/>
+      <c r="W44" s="11" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
       <c r="X44" s="10" t="n"/>
       <c r="Y44" s="10" t="n"/>
       <c r="Z44" s="12" t="n"/>
@@ -2556,7 +2569,7 @@
       <c r="AB44" s="10" t="n"/>
       <c r="AC44" s="11" t="inlineStr">
         <is>
-          <t>11,945</t>
+          <t>108</t>
         </is>
       </c>
       <c r="AD44" s="10" t="n"/>
@@ -2567,14 +2580,22 @@
     <row r="45" ht="17.01" customHeight="1">
       <c r="F45" s="9" t="n"/>
       <c r="G45" s="10" t="n"/>
-      <c r="H45" s="10" t="n"/>
+      <c r="H45" s="11" t="inlineStr">
+        <is>
+          <t>沖縄県</t>
+        </is>
+      </c>
       <c r="I45" s="10" t="n"/>
       <c r="J45" s="10" t="n"/>
       <c r="K45" s="10" t="n"/>
       <c r="L45" s="10" t="n"/>
       <c r="M45" s="12" t="n"/>
       <c r="N45" s="10" t="n"/>
-      <c r="O45" s="10" t="n"/>
+      <c r="O45" s="11" t="inlineStr">
+        <is>
+          <t>398</t>
+        </is>
+      </c>
       <c r="P45" s="10" t="n"/>
       <c r="Q45" s="10" t="n"/>
       <c r="R45" s="10" t="n"/>
@@ -2582,172 +2603,196 @@
       <c r="T45" s="10" t="n"/>
       <c r="U45" s="10" t="n"/>
       <c r="V45" s="10" t="n"/>
-      <c r="W45" s="10" t="n"/>
+      <c r="W45" s="11" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
       <c r="X45" s="10" t="n"/>
       <c r="Y45" s="10" t="n"/>
       <c r="Z45" s="12" t="n"/>
       <c r="AA45" s="10" t="n"/>
       <c r="AB45" s="10" t="n"/>
-      <c r="AC45" s="10" t="n"/>
+      <c r="AC45" s="11" t="inlineStr">
+        <is>
+          <t>127</t>
+        </is>
+      </c>
       <c r="AD45" s="10" t="n"/>
       <c r="AE45" s="10" t="n"/>
       <c r="AF45" s="10" t="n"/>
       <c r="AG45" s="13" t="n"/>
     </row>
     <row r="46" ht="17.01" customHeight="1">
-      <c r="F46" s="14" t="n"/>
-      <c r="G46" s="15" t="n"/>
-      <c r="H46" s="15" t="n"/>
-      <c r="I46" s="15" t="n"/>
-      <c r="J46" s="15" t="n"/>
-      <c r="K46" s="15" t="n"/>
-      <c r="L46" s="15" t="n"/>
+      <c r="F46" s="9" t="n"/>
+      <c r="G46" s="10" t="n"/>
+      <c r="H46" s="10" t="n"/>
+      <c r="I46" s="11" t="inlineStr">
+        <is>
+          <t>合計</t>
+        </is>
+      </c>
+      <c r="J46" s="10" t="n"/>
+      <c r="K46" s="10" t="n"/>
+      <c r="L46" s="10" t="n"/>
       <c r="M46" s="12" t="n"/>
-      <c r="N46" s="15" t="n"/>
-      <c r="O46" s="15" t="n"/>
-      <c r="P46" s="15" t="n"/>
-      <c r="Q46" s="15" t="n"/>
-      <c r="R46" s="15" t="n"/>
+      <c r="N46" s="10" t="n"/>
+      <c r="O46" s="11" t="inlineStr">
+        <is>
+          <t>37,992</t>
+        </is>
+      </c>
+      <c r="P46" s="10" t="n"/>
+      <c r="Q46" s="10" t="n"/>
+      <c r="R46" s="10" t="n"/>
       <c r="S46" s="12" t="n"/>
-      <c r="T46" s="15" t="n"/>
-      <c r="U46" s="15" t="n"/>
-      <c r="V46" s="15" t="n"/>
-      <c r="W46" s="15" t="n"/>
-      <c r="X46" s="15" t="n"/>
-      <c r="Y46" s="15" t="n"/>
+      <c r="T46" s="10" t="n"/>
+      <c r="U46" s="10" t="n"/>
+      <c r="V46" s="11" t="inlineStr">
+        <is>
+          <t>1,610</t>
+        </is>
+      </c>
+      <c r="W46" s="10" t="n"/>
+      <c r="X46" s="10" t="n"/>
+      <c r="Y46" s="10" t="n"/>
       <c r="Z46" s="12" t="n"/>
-      <c r="AA46" s="15" t="n"/>
-      <c r="AB46" s="15" t="n"/>
-      <c r="AC46" s="15" t="n"/>
-      <c r="AD46" s="15" t="n"/>
-      <c r="AE46" s="15" t="n"/>
-      <c r="AF46" s="15" t="n"/>
-      <c r="AG46" s="16" t="n"/>
+      <c r="AA46" s="10" t="n"/>
+      <c r="AB46" s="10" t="n"/>
+      <c r="AC46" s="11" t="inlineStr">
+        <is>
+          <t>11,945</t>
+        </is>
+      </c>
+      <c r="AD46" s="10" t="n"/>
+      <c r="AE46" s="10" t="n"/>
+      <c r="AF46" s="10" t="n"/>
+      <c r="AG46" s="13" t="n"/>
     </row>
     <row r="47" ht="17.01" customHeight="1">
-      <c r="F47" s="14" t="n"/>
-      <c r="G47" s="15" t="n"/>
-      <c r="H47" s="15" t="n"/>
-      <c r="I47" s="15" t="n"/>
-      <c r="J47" s="15" t="n"/>
-      <c r="K47" s="15" t="n"/>
-      <c r="L47" s="15" t="n"/>
+      <c r="F47" s="9" t="n"/>
+      <c r="G47" s="10" t="n"/>
+      <c r="H47" s="10" t="n"/>
+      <c r="I47" s="10" t="n"/>
+      <c r="J47" s="10" t="n"/>
+      <c r="K47" s="10" t="n"/>
+      <c r="L47" s="10" t="n"/>
       <c r="M47" s="12" t="n"/>
-      <c r="N47" s="15" t="n"/>
-      <c r="O47" s="15" t="n"/>
-      <c r="P47" s="15" t="n"/>
-      <c r="Q47" s="15" t="n"/>
-      <c r="R47" s="15" t="n"/>
+      <c r="N47" s="10" t="n"/>
+      <c r="O47" s="10" t="n"/>
+      <c r="P47" s="10" t="n"/>
+      <c r="Q47" s="10" t="n"/>
+      <c r="R47" s="10" t="n"/>
       <c r="S47" s="12" t="n"/>
-      <c r="T47" s="15" t="n"/>
-      <c r="U47" s="15" t="n"/>
-      <c r="V47" s="15" t="n"/>
-      <c r="W47" s="15" t="n"/>
-      <c r="X47" s="15" t="n"/>
-      <c r="Y47" s="15" t="n"/>
+      <c r="T47" s="10" t="n"/>
+      <c r="U47" s="10" t="n"/>
+      <c r="V47" s="10" t="n"/>
+      <c r="W47" s="10" t="n"/>
+      <c r="X47" s="10" t="n"/>
+      <c r="Y47" s="10" t="n"/>
       <c r="Z47" s="12" t="n"/>
-      <c r="AA47" s="15" t="n"/>
-      <c r="AB47" s="15" t="n"/>
-      <c r="AC47" s="15" t="n"/>
-      <c r="AD47" s="15" t="n"/>
-      <c r="AE47" s="15" t="n"/>
-      <c r="AF47" s="15" t="n"/>
-      <c r="AG47" s="16" t="n"/>
+      <c r="AA47" s="10" t="n"/>
+      <c r="AB47" s="10" t="n"/>
+      <c r="AC47" s="10" t="n"/>
+      <c r="AD47" s="10" t="n"/>
+      <c r="AE47" s="10" t="n"/>
+      <c r="AF47" s="10" t="n"/>
+      <c r="AG47" s="13" t="n"/>
     </row>
     <row r="48" ht="17.01" customHeight="1">
-      <c r="F48" s="17" t="n"/>
-      <c r="G48" s="17" t="n"/>
-      <c r="H48" s="17" t="n"/>
-      <c r="I48" s="17" t="n"/>
-      <c r="J48" s="17" t="n"/>
-      <c r="K48" s="17" t="n"/>
-      <c r="L48" s="17" t="n"/>
-      <c r="M48" s="17" t="n"/>
-      <c r="N48" s="17" t="n"/>
-      <c r="O48" s="17" t="n"/>
-      <c r="P48" s="17" t="n"/>
-      <c r="Q48" s="17" t="n"/>
-      <c r="R48" s="17" t="n"/>
-      <c r="S48" s="17" t="n"/>
-      <c r="T48" s="17" t="n"/>
-      <c r="U48" s="17" t="n"/>
-      <c r="V48" s="17" t="n"/>
-      <c r="W48" s="17" t="n"/>
-      <c r="X48" s="17" t="n"/>
-      <c r="Y48" s="17" t="n"/>
-      <c r="Z48" s="17" t="n"/>
-      <c r="AA48" s="17" t="n"/>
-      <c r="AB48" s="17" t="n"/>
-      <c r="AC48" s="17" t="n"/>
-      <c r="AD48" s="17" t="n"/>
-      <c r="AE48" s="17" t="n"/>
-      <c r="AF48" s="17" t="n"/>
-      <c r="AG48" s="17" t="n"/>
+      <c r="F48" s="7" t="n"/>
+      <c r="G48" s="7" t="n"/>
+      <c r="H48" s="7" t="n"/>
+      <c r="I48" s="7" t="n"/>
+      <c r="J48" s="7" t="n"/>
+      <c r="K48" s="7" t="n"/>
+      <c r="L48" s="7" t="n"/>
+      <c r="M48" s="7" t="n"/>
+      <c r="N48" s="7" t="n"/>
+      <c r="O48" s="7" t="n"/>
+      <c r="P48" s="7" t="n"/>
+      <c r="Q48" s="7" t="n"/>
+      <c r="R48" s="7" t="n"/>
+      <c r="S48" s="7" t="n"/>
+      <c r="T48" s="7" t="n"/>
+      <c r="U48" s="7" t="n"/>
+      <c r="V48" s="7" t="n"/>
+      <c r="W48" s="7" t="n"/>
+      <c r="X48" s="7" t="n"/>
+      <c r="Y48" s="7" t="n"/>
+      <c r="Z48" s="7" t="n"/>
+      <c r="AA48" s="7" t="n"/>
+      <c r="AB48" s="7" t="n"/>
+      <c r="AC48" s="7" t="n"/>
+      <c r="AD48" s="7" t="n"/>
+      <c r="AE48" s="7" t="n"/>
+      <c r="AF48" s="7" t="n"/>
+      <c r="AG48" s="7" t="n"/>
     </row>
     <row r="49" ht="17.01" customHeight="1">
-      <c r="F49" s="18" t="n"/>
-      <c r="G49" s="18" t="n"/>
-      <c r="H49" s="18" t="n"/>
-      <c r="I49" s="18" t="n"/>
-      <c r="J49" s="18" t="n"/>
-      <c r="K49" s="18" t="n"/>
-      <c r="L49" s="18" t="n"/>
-      <c r="M49" s="18" t="n"/>
-      <c r="N49" s="18" t="n"/>
-      <c r="O49" s="18" t="n"/>
-      <c r="P49" s="18" t="n"/>
-      <c r="Q49" s="18" t="n"/>
-      <c r="R49" s="18" t="n"/>
-      <c r="S49" s="18" t="n"/>
-      <c r="T49" s="18" t="n"/>
-      <c r="U49" s="18" t="n"/>
-      <c r="V49" s="18" t="n"/>
-      <c r="W49" s="18" t="n"/>
-      <c r="X49" s="18" t="n"/>
-      <c r="Y49" s="18" t="n"/>
-      <c r="Z49" s="18" t="n"/>
-      <c r="AA49" s="18" t="n"/>
-      <c r="AB49" s="18" t="n"/>
-      <c r="AC49" s="18" t="n"/>
-      <c r="AD49" s="18" t="n"/>
-      <c r="AE49" s="18" t="n"/>
-      <c r="AF49" s="18" t="n"/>
-      <c r="AG49" s="18" t="n"/>
+      <c r="F49" s="7" t="n"/>
+      <c r="G49" s="7" t="n"/>
+      <c r="H49" s="7" t="n"/>
+      <c r="I49" s="7" t="n"/>
+      <c r="J49" s="7" t="n"/>
+      <c r="K49" s="7" t="n"/>
+      <c r="L49" s="7" t="n"/>
+      <c r="M49" s="7" t="n"/>
+      <c r="N49" s="7" t="n"/>
+      <c r="O49" s="7" t="n"/>
+      <c r="P49" s="7" t="n"/>
+      <c r="Q49" s="7" t="n"/>
+      <c r="R49" s="7" t="n"/>
+      <c r="S49" s="7" t="n"/>
+      <c r="T49" s="7" t="n"/>
+      <c r="U49" s="7" t="n"/>
+      <c r="V49" s="7" t="n"/>
+      <c r="W49" s="7" t="n"/>
+      <c r="X49" s="7" t="n"/>
+      <c r="Y49" s="7" t="n"/>
+      <c r="Z49" s="7" t="n"/>
+      <c r="AA49" s="7" t="n"/>
+      <c r="AB49" s="7" t="n"/>
+      <c r="AC49" s="7" t="n"/>
+      <c r="AD49" s="7" t="n"/>
+      <c r="AE49" s="7" t="n"/>
+      <c r="AF49" s="7" t="n"/>
+      <c r="AG49" s="7" t="n"/>
     </row>
     <row r="50" ht="17.01" customHeight="1">
-      <c r="F50" s="18" t="n"/>
-      <c r="G50" s="18" t="n"/>
-      <c r="H50" s="18" t="n"/>
-      <c r="I50" s="18" t="n"/>
-      <c r="J50" s="18" t="n"/>
-      <c r="K50" s="18" t="n"/>
-      <c r="L50" s="18" t="n"/>
-      <c r="M50" s="18" t="n"/>
-      <c r="N50" s="18" t="n"/>
-      <c r="O50" s="18" t="n"/>
-      <c r="P50" s="18" t="n"/>
-      <c r="Q50" s="18" t="n"/>
-      <c r="R50" s="18" t="n"/>
-      <c r="S50" s="18" t="n"/>
-      <c r="T50" s="18" t="n"/>
-      <c r="U50" s="18" t="n"/>
-      <c r="V50" s="18" t="n"/>
-      <c r="W50" s="18" t="n"/>
-      <c r="X50" s="18" t="n"/>
-      <c r="Y50" s="18" t="n"/>
-      <c r="Z50" s="18" t="n"/>
-      <c r="AA50" s="18" t="n"/>
-      <c r="AB50" s="18" t="n"/>
-      <c r="AC50" s="18" t="n"/>
-      <c r="AD50" s="18" t="n"/>
-      <c r="AE50" s="18" t="n"/>
-      <c r="AF50" s="18" t="n"/>
-      <c r="AG50" s="18" t="n"/>
+      <c r="F50" s="7" t="n"/>
+      <c r="G50" s="7" t="n"/>
+      <c r="H50" s="7" t="n"/>
+      <c r="I50" s="7" t="n"/>
+      <c r="J50" s="7" t="n"/>
+      <c r="K50" s="7" t="n"/>
+      <c r="L50" s="7" t="n"/>
+      <c r="M50" s="7" t="n"/>
+      <c r="N50" s="7" t="n"/>
+      <c r="O50" s="7" t="n"/>
+      <c r="P50" s="7" t="n"/>
+      <c r="Q50" s="7" t="n"/>
+      <c r="R50" s="7" t="n"/>
+      <c r="S50" s="7" t="n"/>
+      <c r="T50" s="7" t="n"/>
+      <c r="U50" s="7" t="n"/>
+      <c r="V50" s="7" t="n"/>
+      <c r="W50" s="7" t="n"/>
+      <c r="X50" s="7" t="n"/>
+      <c r="Y50" s="7" t="n"/>
+      <c r="Z50" s="7" t="n"/>
+      <c r="AA50" s="7" t="n"/>
+      <c r="AB50" s="7" t="n"/>
+      <c r="AC50" s="7" t="n"/>
+      <c r="AD50" s="7" t="n"/>
+      <c r="AE50" s="7" t="n"/>
+      <c r="AF50" s="7" t="n"/>
+      <c r="AG50" s="7" t="n"/>
     </row>
     <row r="51" ht="17.01" customHeight="1"/>
     <row r="52" ht="17.01" customHeight="1"/>
   </sheetData>
-  <pageMargins left="0.47" right="0.47" top="0.41" bottom="0.41" header="0" footer="0"/>
+  <pageMargins left="0.47" right="0.47" top="0.41" bottom="0.41" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9"/>
 </worksheet>
 </file>
</xml_diff>